<commit_message>
fix: set AI-Startklar attendance print area
</commit_message>
<xml_diff>
--- a/deliverables/ai-startklar/vertrieb/13-teilnahmeliste.xlsx
+++ b/deliverables/ai-startklar/vertrieb/13-teilnahmeliste.xlsx
@@ -2,8 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teilnahmeliste" sheetId="1" r:id="R16364ae785b24b04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teilnahmeliste" sheetId="1" r:id="R8a2f47878e194c98"/>
   </x:sheets>
+  <x:definedNames>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Teilnahmeliste'!$A$1:$E$25</x:definedName>
+  </x:definedNames>
 </x:workbook>
 </file>
 

</xml_diff>